<commit_message>
docs(assets): rewrite v6 xlsx in non-developer-friendly Korean
용어 정리·문체 평이화:
- "redundant" -> "생략", "prefix" -> "종류 약자/앞 약자"
- "suffix" -> "뒤 약자", "vocab" -> "정해진 단어 모음/약자"
- "normalization" -> "통일된 형식으로 변환"
- "deterministic" -> "정해진 순서대로"
- "ad-hoc" -> "그때그때 임의로"
- "kind prefix" -> "종류 표시 약자"
- "sibling vocab" -> "형제 노드 한 글자"

Overview 시트에 "이 문서를 읽기 전에 — 용어 안내" 섹션 신설:
원본 에셋·인스턴스·씬 트리·앞 약자/뒤 약자·Vocab·T1/T2/T3
6개 용어를 비개발자 친화적으로 풀이.

각 시트의 제목·노트·표 헤더·설명 행을 평이한 한국어로 재작성.
규칙 자체(약자·형식·예시)는 변경 없음.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/doc/assets/MakeNamingConvention_v6.xlsx
+++ b/doc/assets/MakeNamingConvention_v6.xlsx
@@ -496,13 +496,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -523,333 +523,424 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>[ 핵심 원칙 ]</t>
+          <t>[ 이 문서를 읽기 전에 — 용어 안내 ]</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>원칙</t>
+          <t>용어</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>설명</t>
+          <t>쉽게 풀어 쓰기</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>1. 컨텍스트별 형식 분리</t>
+          <t>원본 에셋 (Source Asset)</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>T1 파일 탐색기 / T2 Make Editor / T3 JSON·grep — 각 컨텍스트 최적화</t>
+          <t>모델러·디자이너가 만들어 전달하는 원본 파일. 예: .fbx, .png, .wav</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>2. 인스턴스명에 prefix 없음</t>
+          <t>인스턴스 (Instance)</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Make Editor 의 타입 아이콘이 종류를 시각적으로 알려주므로 redundant</t>
+          <t>Make Editor 안에 배치된 객체. 원본 파일을 씬에 가져다 놓은 것</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>3. 트리 컨텍스트 활용</t>
+          <t>씬 트리 (Scene Tree)</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>부모-자식 위계가 트리에 명시 → 자식 이름은 짧게</t>
+          <t>Make Editor 의 왼쪽 계층 구조. 부모-자식 관계로 객체가 묶여 있음</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>4. 단일 `_` 통일</t>
+          <t>앞 약자 / 뒤 약자</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>이중 `__` 폐지, 하이픈 명시 금지</t>
+          <t>이름 맨 앞 또는 맨 뒤에 붙는 짧은 표시 글자 (예: GNB_, _On)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>5. Vocab 축약</t>
+          <t>Vocab (정해진 단어 모음)</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>State·Action·Direction 모두 축약형 (3-letter 또는 단문자)</t>
+          <t>허용된 단어 목록. 이 안에서만 골라 써야 함</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>6. 자가설명은 시스템 파생만</t>
+          <t>T1 / T2 / T3</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>사용자 미편집 객체 (T3) 만 prefix 보존 — AI grep·로그 안전</t>
+          <t>이 문서가 정한 세 단계: 원본 파일 / 배치된 인스턴스 / 자동 생성 객체</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>[ 3-Tier 모델 ]</t>
+          <t>[ 이 규칙이 따르는 6가지 큰 원칙 ]</t>
         </is>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Tier</t>
+          <t>원칙</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>이름</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>컨텍스트</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>형식</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>예시</t>
+          <t>쉬운 설명</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>1. 어디서 보는지에 따라 다르게</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Source Asset</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>파일시스템 (OS 탐색기)</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>PascalCase + 확장자 + 카테고리 토큰</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>GlassBottle_v01.fbx, GNB_Active.png, BGM_Tutorial_01.wav</t>
+          <t>OS 파일 탐색기 / Make Editor / 코드 검색 — 각자 보기 좋은 모양이 다름</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>2. Make Editor 안의 이름은 짧게</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Instance</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Make Editor 트리</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>PascalCase, prefix 없음, 단일 _</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>GNB_Act, BtnStart, Cupcake, RotationPanel/L</t>
+          <t>Make Editor 가 이미 아이콘으로 종류를 알려주므로 이름에 종류 표시 약자는 생략</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>3. 부모-자식 관계는 트리로 표현</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>System-Derived</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>머티리얼·중간 mesh·texture object</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>lower_snake_case + 3-letter kind prefix</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>mat_unlit_opaque, tex_cupcake_albedo</t>
+          <t>부모 이름을 자식 이름에 반복해 적지 않음 — 트리가 이미 알려주니까</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>4. 구분 기호는 언더바 _ 하나만</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>이중 언더바 __ 와 하이픈 - 은 모두 사용 금지</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>[ 시트 안내 ]</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>시트</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>내용</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Overview</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>본 시트 — 원칙·3-Tier 요약</t>
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>5. 약자로 짧게 쓰기</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>상태·동작·방향 모두 정해진 짧은 약자로 (3글자 또는 1글자)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>6. 자동 생성 객체만 종류 표시</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>사람이 직접 안 만지는 머티리얼·중간 노드만 mat_ 같은 약자 유지</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>T1 Source</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>파일시스템 원본 에셋 명명 규칙 (FBX·PNG·WAV·MP4·Font)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>T2 Instance</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Make Editor 인스턴스 명명 규칙 + Family/State/Direction Vocab</t>
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>[ 3단계 (T1 / T2 / T3) ]</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>단계</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>무엇인지</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>어디서 보이는지</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>쓰는 모양</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>예시</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>T3 Derived</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>시스템 파생 객체 명명 규칙 (머티리얼 등)</t>
+          <t>원본 파일</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>OS 파일 탐색기에서 보임</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>PascalCase + 확장자 + (필요 시) 카테고리 약자</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>GlassBottle_v01.fbx, GNB_Active.png, BGM_Tutorial_01.wav</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Animation</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>애니메이션 클립 명명 규칙 + Action Vocab</t>
+          <t>Make Editor 인스턴스</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Make Editor 의 씬 트리에서 보임</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>PascalCase, 종류 약자 없음, 언더바 하나만</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>GNB_Act, BtnStart, Cupcake, RotationPanel/L</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>자동 생성 객체</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>사람이 직접 안 만지는 머티리얼·중간 노드</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>소문자_snake_case + 3글자 종류 약자</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>mat_unlit_opaque, tex_cupcake_albedo</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>[ 시트 안내 ]</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>시트</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>내용</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>이 시트 — 큰 원칙과 3단계 요약</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>T1 Source</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>원본 파일 이름 규칙 (3D 모델·이미지·소리·영상·폰트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>T2 Instance</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Make Editor 인스턴스 이름 규칙 + 자주 쓰는 단어 모음</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>T3 Derived</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>자동으로 만들어지는 객체 이름 규칙</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>애니메이션 이름 규칙 + 동작·방향 약자 모음</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
           <t>Vocab Tables</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>UI Family / State / Direction / Action / Audio·Video 카테고리 통합</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>약자·단어 모음 한눈에 보기</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>Examples</t>
         </is>
       </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>실측 파일(Make Templete_20260512.make) 안티패턴 → v6 변환 가이드</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>실제 파일을 v6 규칙으로 바꾼 비교표</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>Checklist</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>익스포트 전 검증 체크리스트</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>내보내기 전에 확인할 항목 (체크리스트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>Anti-Patterns</t>
         </is>
       </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>금지 패턴 일람</t>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>이렇게 쓰면 안 되는 예시</t>
         </is>
       </c>
     </row>
@@ -875,45 +966,45 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>T1 — Source Asset (Filesystem)</t>
+          <t>T1 — 원본 파일 이름 규칙</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>모델러·아티스트가 납품 또는 작업 디렉토리에 두는 원본 파일. PascalCase + 확장자. 확장자가 타입을 선언하므로 kind prefix 불필요. 모호한 타입(PNG/WAV/MP4) 만 카테고리·Role 토큰 사용.</t>
+          <t>모델러·디자이너가 만들어서 전달하는 원본 파일(작업 폴더에 있는 파일)에 적용. PascalCase 로 쓰고 확장자(.fbx, .png 등)를 붙임. 확장자가 종류를 알려주므로 이름 앞에 종류 약자(mdl_ 등)는 생략. 단, PNG·WAV·MP4 처럼 같은 확장자가 여러 용도로 쓰이는 경우에만 카테고리 약자를 이름 안에 넣음.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>[ Global Rules ]</t>
+          <t>[ 공통 규칙 ]</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Rule</t>
+          <t>규칙</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>✅ Correct</t>
+          <t>✅ 이렇게 쓰세요</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>❌ Incorrect</t>
+          <t>❌ 이렇게 쓰지 마세요</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>공백 없음</t>
+          <t>이름에 공백을 넣지 않는다</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -930,7 +1021,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>구분자 _ 만 (하이픈 금지)</t>
+          <t>구분 기호는 언더바 _ 만 (하이픈 - 금지)</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -947,7 +1038,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>토큰별 PascalCase</t>
+          <t>단어마다 첫 글자는 대문자 (PascalCase)</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -964,7 +1055,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Variant 2자리 고정</t>
+          <t>변형 번호는 두 자리로 통일</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -981,7 +1072,7 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Version v + 2자리 (옵션)</t>
+          <t>버전은 v + 두 자리 (선택 사항)</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -998,7 +1089,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>중복 타입 토큰 금지</t>
+          <t>확장자가 알려주는 종류를 이름에 또 적지 않는다</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -1015,7 +1106,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>영문 전용</t>
+          <t>영문으로만 적기 (한글 파일명 금지)</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -1032,33 +1123,33 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>[ 타입별 규칙 ]</t>
+          <t>[ 파일 종류별 규칙 ]</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>■ 3D Model (.fbx)</t>
+          <t>■ 3D 모델 (.fbx)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>확장자 .fbx 가 타입 선언. 이름에 타입 토큰 박지 말 것. 자식 부위는 부모 이름 포함.</t>
+          <t>확장자 .fbx 가 "3D 모델"이라는 종류를 알려줍니다. 이름에 또 적지 마세요. 자식 부품을 별도 파일로 보낼 때는 부모 이름을 함께 적어 어떤 모델의 부품인지 알 수 있게 하세요.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>파일명</t>
+          <t>파일 이름</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>용도</t>
+          <t>쓰임새</t>
         </is>
       </c>
     </row>
@@ -1070,7 +1161,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>루트 모델</t>
+          <t>기본 모델</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1173,7 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>버전 업데이트</t>
+          <t>수정된 버전 (v02)</t>
         </is>
       </c>
     </row>
@@ -1094,7 +1185,7 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>State 변형</t>
+          <t>다른 형태 (뚜껑 열린 버전)</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1197,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>자식 부위 — 부모 이름 포함</t>
+          <t>자식 부품 — 부모 이름 포함</t>
         </is>
       </c>
     </row>
@@ -1118,14 +1209,14 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>자식 부위</t>
+          <t>자식 부품</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>■ Image — UI Sprite (.png/.jpg)</t>
+          <t>■ 이미지 — UI 스프라이트 (.png/.jpg)</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1235,7 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Family + Asset + State</t>
+          <t>종류 약자(Family) + 이름 + 상태</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
@@ -1156,7 +1247,7 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Family 단독 사용 OK (단일 자산일 때)</t>
+          <t>Family 만으로 충분할 때는 단독 사용 OK</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -1168,7 +1259,7 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>State suffix 는 v6 축약 (Def/Prs/On/Off/Sel)</t>
+          <t>상태 약자는 정해진 5개 안에서만 사용</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
@@ -1180,7 +1271,7 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Direction 은 단문자 suffix</t>
+          <t>방향은 한 글자로 (L/R/U/D)</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -1192,21 +1283,21 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>■ Image — 3D Texture (.png)</t>
+          <t>■ 이미지 — 3D 텍스처 (.png)</t>
         </is>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Role 토큰 필수 — PNG 는 UI 와 텍스처 둘 다이므로 확장자만으론 분간 불가. v&lt;NN&gt; 미사용 (아트 에셋).</t>
+          <t>용도 약자(Role)를 반드시 넣으세요. PNG 는 UI 와 3D 텍스처 둘 다에 쓰여서 확장자만으론 어디 쓰이는지 알 수 없기 때문입니다. 텍스처는 "버전 표시 _v01" 을 쓰지 않습니다 (디자이너가 자유롭게 갱신하는 아트 자산이므로).</t>
         </is>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>Token</t>
+          <t>약자</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -1228,7 +1319,7 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>UI 스프라이트</t>
+          <t>UI 스프라이트 (버튼·아이콘 등)</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
@@ -1245,7 +1336,7 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Albedo / Base Color</t>
+          <t>Albedo / 기본 색상 텍스처</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
@@ -1262,7 +1353,7 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Normal Map</t>
+          <t>Normal Map (표면 굴곡)</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
@@ -1279,7 +1370,7 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Roughness</t>
+          <t>Roughness (거칠기)</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
@@ -1296,7 +1387,7 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Metallic</t>
+          <t>Metallic (금속성)</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
@@ -1313,7 +1404,7 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Emission</t>
+          <t>Emission (자체 발광)</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
@@ -1330,7 +1421,7 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>Mask</t>
+          <t>Mask (마스킹)</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
@@ -1347,7 +1438,7 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Ambient Occlusion</t>
+          <t>Ambient Occlusion (음영)</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
@@ -1359,26 +1450,26 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>■ Audio (.wav / .mp3)</t>
+          <t>■ 소리 (.wav / .mp3)</t>
         </is>
       </c>
     </row>
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>&lt;Category&gt;_&lt;Description&gt;_&lt;NN&gt;.&lt;ext&gt; — 카테고리·description 사이 _ 삽입 (v6).</t>
+          <t>형식: &lt;카테고리&gt;_&lt;설명&gt;_&lt;번호&gt;.확장자. 카테고리 약자와 설명 사이에 언더바 _ 를 한 번 넣습니다.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="22" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>카테고리</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>풀이</t>
+          <t>의미</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
@@ -1395,7 +1486,7 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>Background Music</t>
+          <t>배경 음악</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
@@ -1412,7 +1503,7 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Sound Effect (UI 클릭·완료음·경고)</t>
+          <t>효과음 (버튼 클릭·완료음·경고음 등)</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
@@ -1429,7 +1520,7 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Narration / 더빙 (구 VO)</t>
+          <t>내레이션·더빙 (이전 이름: VO)</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
@@ -1441,19 +1532,19 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>■ Video (.mp4)</t>
+          <t>■ 영상 (.mp4)</t>
         </is>
       </c>
     </row>
     <row r="55" ht="22" customHeight="1">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>카테고리</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>풀이</t>
+          <t>의미</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -1470,7 +1561,7 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>Cutscene (시네마틱·서사 영상)</t>
+          <t>컷씬 (서사·시네마틱 영상)</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
@@ -1487,7 +1578,7 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>Tutorial (단계별 설명)</t>
+          <t>튜토리얼 (단계별 설명 영상)</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
@@ -1504,7 +1595,7 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>Looping background video</t>
+          <t>반복 재생되는 배경 영상</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
@@ -1521,7 +1612,7 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>Intro sequence</t>
+          <t>콘텐츠 시작 인트로</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
@@ -1538,7 +1629,7 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>Outro sequence</t>
+          <t>콘텐츠 끝 아웃트로</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
@@ -1550,19 +1641,19 @@
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>■ Font (.ttf / .otf)</t>
+          <t>■ 폰트 (.ttf / .otf)</t>
         </is>
       </c>
     </row>
     <row r="63" ht="22" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>파일명</t>
+          <t>파일 이름</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>비고</t>
+          <t>구성</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1665,7 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>본체 + Weight</t>
+          <t>폰트 이름 + 굵기</t>
         </is>
       </c>
     </row>
@@ -1614,53 +1705,53 @@
   <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>T2 — Instance (Make Editor visible)</t>
+          <t>T2 — Make Editor 인스턴스 이름 규칙</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Make Editor 트리에 노출되는 사용자 직접 명명 노드. 트리 옆 타입 아이콘이 종류를 시각화하므로 kind prefix 폐지. 부모-자식 트리가 위계를 표현하므로 자식 이름은 짧게.</t>
+          <t>Make Editor 의 씬 트리에 보이는, 사용자가 직접 이름을 짓는 객체입니다. 트리 옆 아이콘이 종류를 알려주므로 이름에 종류 약자(mdl_, img_ 같은 것) 는 생략합니다. 부모-자식 관계는 트리가 이미 보여주므로 자식 이름은 짧게 적습니다.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>[ Core Rules ]</t>
+          <t>[ 가장 중요한 규칙 ]</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Rule</t>
+          <t>규칙</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>✅ Correct</t>
+          <t>✅ 이렇게 쓰세요</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>❌ Incorrect</t>
+          <t>❌ 이렇게 쓰지 마세요</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>PascalCase 토큰</t>
+          <t>단어마다 첫 글자 대문자 (PascalCase)</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -1677,7 +1768,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Prefix 없음 (T2 한정)</t>
+          <t>종류 약자 생략 (T2 에서만 해당)</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -1694,7 +1785,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>단일 _ 만</t>
+          <t>언더바 _ 하나만 사용</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -1711,7 +1802,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>확장자 없음</t>
+          <t>이름 끝에 확장자 안 붙이기</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1728,24 +1819,24 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>닫힌 sibling vocab 단문자 OK</t>
+          <t>정해진 4방향 자식은 한 글자로 OK</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>RotationPanel/L /R /U /D</t>
+          <t>RotationPanel 아래에 L /R /U /D</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>(자유 명명 sibling 에선 금지)</t>
+          <t>(자유롭게 이름 짓는 형제 노드 사이에선 금지)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>자유 명명 sibling 의미 슬러그</t>
+          <t>자유 명명일 때는 의미 있는 이름</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -1755,28 +1846,28 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>R, Z (모호)</t>
+          <t>R, Z (무슨 뜻인지 모름)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>[ Syntax ]</t>
+          <t>[ 이름 짜는 순서 ]</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>&lt;Family&gt;&lt;Asset&gt;[_&lt;Direction&gt;][_&lt;State&gt;]</t>
+          <t>&lt;종류 약자&gt;&lt;고유 이름&gt;[_&lt;방향&gt;][_&lt;상태&gt;]</t>
         </is>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>토큰</t>
+          <t>부분</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -1793,12 +1884,12 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Family</t>
+          <t>종류 약자 (Family)</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>UI Family Vocab (권장, 선택)</t>
+          <t>어떤 UI 인지 알려주는 짧은 약자 (선택 사항, 권장)</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -1810,12 +1901,12 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Asset</t>
+          <t>고유 이름</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>자산 슬러그 (PascalCase)</t>
+          <t>이 객체만의 이름 (PascalCase)</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -1827,12 +1918,12 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Direction</t>
+          <t>방향</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>방향 단문자 (해당 시)</t>
+          <t>방향 정보가 있을 때 한 글자로</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -1844,12 +1935,12 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>State</t>
+          <t>상태</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>3-letter 축약</t>
+          <t>3글자 약자</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -1876,7 +1967,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
   </cols>
@@ -1884,42 +1975,42 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>T3 — System-Derived Identifier</t>
+          <t>T3 — 자동 생성 객체 이름 규칙</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>사용자가 직접 명명하지 않는 객체 (머티리얼·중간 mesh 노드·texture object). AI grep·로그 단독 노출 빈도 높음 → prefix 유지가 가치 큼. 시스템 자동 파생 (Tier C) 이라 사용자 명명 부담 0.</t>
+          <t>사용자가 직접 이름을 짓지 않는 객체입니다 (머티리얼·중간 mesh 노드·텍스처 등). 시스템이 자동으로 만들고, 사용자는 머티리얼 패널 등에서 가끔 본다는 정도. 이런 객체는 이름이 단독으로 로그·검색 결과에 나타나므로 종류 약자(mat_, tex_ 등)를 유지해 "이게 뭔지" 알 수 있게 합니다.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>[ Format ]</t>
+          <t>[ 이름 형식 ]</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>&lt;kind&gt;_&lt;asset&gt;[_&lt;component&gt;][_&lt;channel|state&gt;]</t>
+          <t>&lt;종류약자&gt;_&lt;이름&gt;[_&lt;부위&gt;][_&lt;채널 또는 상태&gt;]</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>[ Kind Prefix Table (3-letter) ]</t>
+          <t>[ 종류 약자 (3글자) ]</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Prefix</t>
+          <t>약자</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -1946,7 +2037,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>3D Model (mesh/node)</t>
+          <t>3D 모델 (mesh/node)</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -1968,12 +2059,12 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Material</t>
+          <t>머티리얼 (재질)</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>(논리)</t>
+          <t>(개념상)</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -1990,7 +2081,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Texture (3D input)</t>
+          <t>텍스처 (3D 모델 표면용)</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -2012,7 +2103,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>UI Image (2D)</t>
+          <t>UI 이미지 (2D)</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -2034,7 +2125,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Audio</t>
+          <t>오디오</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -2056,7 +2147,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>비디오</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -2066,7 +2157,7 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>external</t>
+          <t>외부 파일</t>
         </is>
       </c>
     </row>
@@ -2078,12 +2169,12 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Event trigger</t>
+          <t>이벤트 트리거</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>(논리)</t>
+          <t>(개념상)</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -2100,12 +2191,12 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Scene container</t>
+          <t>씬 컨테이너</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>(논리)</t>
+          <t>(개념상)</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
@@ -2122,31 +2213,31 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Generic group</t>
+          <t>일반 그룹</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>(논리)</t>
+          <t>(개념상)</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>empty transform</t>
+          <t>빈 transform</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>[ Auto-Derivation Rule ]</t>
+          <t>[ 자동으로 이름 만드는 방법 ]</t>
         </is>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>케이스</t>
+          <t>상황</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -2163,12 +2254,12 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>일반 mirror</t>
+          <t>기본 (1:1)</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>source 이름의 prefix 만 교체</t>
+          <t>원본 이름의 약자만 바꿔치기</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -2180,12 +2271,12 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>1:N 채널 분기</t>
+          <t>하나의 원본이 여러 곳에 쓰일 때</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>채널 suffix 부착</t>
+          <t>채널 약자를 뒤에 붙임</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -2197,31 +2288,31 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>애니메이션 (v6 별도)</t>
+          <t>애니메이션 (v6 별도 규칙)</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>primary channel target 분석</t>
+          <t>주로 어떤 노드를 움직이는지 분석</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Cupcake_Rot_R (T2 식별자, prefix 없음)</t>
+          <t>Cupcake_Rot_R (T2 이름, 종류 약자 없음)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>[ Texture Channel Suffix Vocab ]</t>
+          <t>[ 텍스처 채널 뒤 약자 ]</t>
         </is>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Suffix</t>
+          <t>뒤 약자</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -2238,7 +2329,7 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Base color / diffuse</t>
+          <t>기본 색상 (Base color / diffuse)</t>
         </is>
       </c>
     </row>
@@ -2250,7 +2341,7 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Normal map</t>
+          <t>표면 굴곡 (Normal map)</t>
         </is>
       </c>
     </row>
@@ -2262,7 +2353,7 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Roughness</t>
+          <t>거칠기</t>
         </is>
       </c>
     </row>
@@ -2274,7 +2365,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Metallic</t>
+          <t>금속성</t>
         </is>
       </c>
     </row>
@@ -2286,7 +2377,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Ambient occlusion</t>
+          <t>음영 (Ambient occlusion)</t>
         </is>
       </c>
     </row>
@@ -2298,7 +2389,7 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Emissive</t>
+          <t>자체 발광</t>
         </is>
       </c>
     </row>
@@ -2310,7 +2401,7 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Height / displacement</t>
+          <t>높낮이 (Height / displacement)</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2413,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Alpha mask</t>
+          <t>투명도 (Alpha mask)</t>
         </is>
       </c>
     </row>
@@ -2334,7 +2425,7 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Occlusion-Roughness-Metallic 합성</t>
+          <t>음영·거칠기·금속성 합쳐 놓은 텍스처</t>
         </is>
       </c>
     </row>
@@ -2356,56 +2447,56 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Animation Naming (v6)</t>
+          <t>애니메이션 이름 규칙 (v6)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>애니메이션은 animations[] 배열에 위치 — 타입이 위치로 선언되므로 prefix 없음. 한 클립이 여러 속성 (rotation/scale/translation/color/opacity) 을 동시에 변경 가능.</t>
+          <t>애니메이션은 "애니메이션 목록"이라는 별도 공간에 들어 있어서 종류 약자가 필요 없습니다. 하나의 애니메이션이 회전·크기·위치·색상·투명도 등 여러 속성을 동시에 바꿀 수 있습니다.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>[ Syntax ]</t>
+          <t>[ 이름 짜는 순서 ]</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>&lt;Target&gt;_&lt;Act1&gt;[_&lt;Dir1&gt;][_&lt;Act2&gt;[_&lt;Dir2&gt;]]...</t>
+          <t>&lt;움직일 대상&gt;_&lt;동작1&gt;[_&lt;방향1&gt;][_&lt;동작2&gt;[_&lt;방향2&gt;]]...</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>다중 속성 순서: Rot → Scl → Mov → Clr → Op (결정론적)</t>
+          <t>여러 동작이 섞일 때 적는 순서: 회전 → 크기 → 이동 → 색상 → 투명도</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>[ Action Vocab ]</t>
+          <t>[ 동작 약자 ]</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Abbr</t>
+          <t>약자</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -2415,7 +2506,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>채널 path</t>
+          <t>어떤 동작인지</t>
         </is>
       </c>
     </row>
@@ -2427,12 +2518,12 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Rotate</t>
+          <t>Rotate (회전)</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>rotation</t>
+          <t>회전축이 바뀜</t>
         </is>
       </c>
     </row>
@@ -2444,12 +2535,12 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Scale</t>
+          <t>Scale (크기)</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>scale</t>
+          <t>크기가 바뀜</t>
         </is>
       </c>
     </row>
@@ -2461,12 +2552,12 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Move</t>
+          <t>Move (이동)</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>translation</t>
+          <t>위치가 바뀜</t>
         </is>
       </c>
     </row>
@@ -2478,12 +2569,12 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Color</t>
+          <t>Color (색상)</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>material color / texture switch</t>
+          <t>재질 색상 / 텍스처 교체</t>
         </is>
       </c>
     </row>
@@ -2495,26 +2586,26 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Opacity</t>
+          <t>Opacity (투명도)</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>alpha</t>
+          <t>투명/불투명 변화</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>[ Compound Short-forms (UX 패턴) ]</t>
+          <t>[ 자주 쓰는 동작 묶음 (한 줄로 줄인 형태) ]</t>
         </is>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Abbr</t>
+          <t>약자</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -2524,7 +2615,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>채널 조합</t>
+          <t>어떤 조합인지</t>
         </is>
       </c>
     </row>
@@ -2536,12 +2627,12 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Zoom In</t>
+          <t>Zoom In (확대)</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Scl + Mov (towards)</t>
+          <t>크기 + 이동 (가까이 오기)</t>
         </is>
       </c>
     </row>
@@ -2553,12 +2644,12 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Zoom Out</t>
+          <t>Zoom Out (축소)</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Scl + Mov (away)</t>
+          <t>크기 + 이동 (멀어지기)</t>
         </is>
       </c>
     </row>
@@ -2570,12 +2661,12 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Fade In</t>
+          <t>Fade In (서서히 나타남)</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Op (0→1)</t>
+          <t>투명도 0→1</t>
         </is>
       </c>
     </row>
@@ -2587,12 +2678,12 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Fade Out</t>
+          <t>Fade Out (서서히 사라짐)</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Op (1→0)</t>
+          <t>투명도 1→0</t>
         </is>
       </c>
     </row>
@@ -2604,12 +2695,12 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Transform (full)</t>
+          <t>Transform (전체 변형)</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Rot + Scl + Mov</t>
+          <t>회전 + 크기 + 이동</t>
         </is>
       </c>
     </row>
@@ -2621,26 +2712,26 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Pop (scale easing)</t>
+          <t>Pop (튕기듯 등장)</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Scl with bounce</t>
+          <t>크기에 바운스 효과</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>[ Direction Vocab (Rot/Mov 에 부속) ]</t>
+          <t>[ 방향 약자 (회전·이동에 함께 사용) ]</t>
         </is>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Abbr</t>
+          <t>약자</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -2657,7 +2748,7 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Left</t>
+          <t>Left (왼쪽)</t>
         </is>
       </c>
     </row>
@@ -2669,7 +2760,7 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>Right (오른쪽)</t>
         </is>
       </c>
     </row>
@@ -2681,7 +2772,7 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Up</t>
+          <t>Up (위)</t>
         </is>
       </c>
     </row>
@@ -2693,7 +2784,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Down</t>
+          <t>Down (아래)</t>
         </is>
       </c>
     </row>
@@ -2705,7 +2796,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Clockwise</t>
+          <t>Clockwise (시계 방향)</t>
         </is>
       </c>
     </row>
@@ -2717,26 +2808,26 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Counter-clockwise</t>
+          <t>Counter-clockwise (반시계 방향)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>[ 실측 7개 default 애니메이션 변환 ]</t>
+          <t>[ 실제 파일의 "new Clip" 7개를 v6 로 바꾼 예 ]</t>
         </is>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>현재 (default)</t>
+          <t>현재 이름 (기본값)</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>채널·path</t>
+          <t>어떤 속성이 바뀌나</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -2748,12 +2839,12 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>new Clip (btn_start, scale)</t>
+          <t>new Clip (btn_start, 크기)</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>scale</t>
+          <t>크기 변화</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
@@ -2765,12 +2856,12 @@
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>new Clip (3D Model, rotation)</t>
+          <t>new Clip (3D Model, 회전)</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>rotation</t>
+          <t>회전</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
@@ -2782,12 +2873,12 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>new Clip1 (3D Model, rotation)</t>
+          <t>new Clip1 (3D Model, 회전)</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>rotation</t>
+          <t>회전</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
@@ -2799,12 +2890,12 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>new Clip2 (3D Model, rotation)</t>
+          <t>new Clip2 (3D Model, 회전)</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>rotation</t>
+          <t>회전</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
@@ -2816,12 +2907,12 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>new Clip3 (3D Model, rotation)</t>
+          <t>new Clip3 (3D Model, 회전)</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>rotation</t>
+          <t>회전</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
@@ -2833,12 +2924,12 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>new Clip4 (3D Model, scale+translation)</t>
+          <t>new Clip4 (3D Model, 크기+이동)</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>scale+translation</t>
+          <t>크기 + 이동</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
@@ -2850,12 +2941,12 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>new Clip5 (3D Model, scale)</t>
+          <t>new Clip5 (3D Model, 크기)</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>scale</t>
+          <t>크기 변화</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
@@ -2867,7 +2958,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>[ 다중 속성 예시 ]</t>
+          <t>[ 여러 속성이 섞인 경우 ]</t>
         </is>
       </c>
     </row>
@@ -2903,7 +2994,7 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>스케일 + 페이드 인</t>
+          <t>크기 변화 + 서서히 나타남</t>
         </is>
       </c>
     </row>
@@ -2915,7 +3006,7 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>전체 변환 + 색상</t>
+          <t>전체 변형 + 색상 변화</t>
         </is>
       </c>
     </row>
@@ -2927,7 +3018,7 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>로고 스케일 + 페이드 아웃</t>
+          <t>로고 크기 변화 + 서서히 사라짐</t>
         </is>
       </c>
     </row>
@@ -2949,28 +3040,28 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Vocabulary Tables — 통합 참조</t>
+          <t>약자·단어 모음 한눈에 보기</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>[ UI Family Vocab (T2 인스턴스용, 권장) ]</t>
+          <t>[ UI 종류 약자 (T2 인스턴스용, 권장) ]</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Family</t>
+          <t>약자</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -2980,7 +3071,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Asset slug</t>
+          <t>이름이 함께 필요한지</t>
         </is>
       </c>
     </row>
@@ -2992,12 +3083,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Global Navigation Bar</t>
+          <t>Global Navigation Bar (전체 메뉴바)</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Asset 불필요 (단독 사용 OK)</t>
+          <t>이름 추가 안 해도 됨</t>
         </is>
       </c>
     </row>
@@ -3009,12 +3100,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Local Navigation Bar</t>
+          <t>Local Navigation Bar (하위 메뉴바)</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Asset 불필요</t>
+          <t>이름 추가 안 해도 됨</t>
         </is>
       </c>
     </row>
@@ -3026,12 +3117,12 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Button (generic)</t>
+          <t>Button (버튼)</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Asset 필수</t>
+          <t>이름 반드시 함께</t>
         </is>
       </c>
     </row>
@@ -3043,12 +3134,12 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Navigation control (prev/next)</t>
+          <t>Navigation control (앞/뒤 이동 버튼)</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Asset 불필요</t>
+          <t>이름 추가 안 해도 됨</t>
         </is>
       </c>
     </row>
@@ -3060,12 +3151,12 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Panel / Background container</t>
+          <t>Panel / Background container (패널·배경판)</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Asset 불필요</t>
+          <t>이름 추가 안 해도 됨</t>
         </is>
       </c>
     </row>
@@ -3077,12 +3168,12 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Icon</t>
+          <t>Icon (아이콘)</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Asset 필수</t>
+          <t>이름 반드시 함께</t>
         </is>
       </c>
     </row>
@@ -3094,12 +3185,12 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Background image</t>
+          <t>Background image (배경 이미지)</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Asset 불필요</t>
+          <t>이름 추가 안 해도 됨</t>
         </is>
       </c>
     </row>
@@ -3111,12 +3202,12 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Logo / Brand mark</t>
+          <t>Logo / Brand mark (로고)</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Asset 불필요</t>
+          <t>이름 추가 안 해도 됨</t>
         </is>
       </c>
     </row>
@@ -3128,12 +3219,12 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Tooltip</t>
+          <t>Tooltip (말풍선·도움말)</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Asset 불필요</t>
+          <t>이름 추가 안 해도 됨</t>
         </is>
       </c>
     </row>
@@ -3145,26 +3236,26 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Text / Label (family, prefix 아님)</t>
+          <t>Text / Label (텍스트·라벨)</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Asset 필수</t>
+          <t>이름 반드시 함께</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>[ State Vocab (3-letter PascalCase) ]</t>
+          <t>[ 상태 약자 (3글자) ]</t>
         </is>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Suffix</t>
+          <t>약자</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -3191,7 +3282,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>기본</t>
+          <t>기본 상태</t>
         </is>
       </c>
     </row>
@@ -3208,7 +3299,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>눌림</t>
+          <t>눌려 있는 상태</t>
         </is>
       </c>
     </row>
@@ -3220,12 +3311,12 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>On (구 Active)</t>
+          <t>On (이전: Active)</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>활성/켜짐</t>
+          <t>켜짐 / 활성 상태</t>
         </is>
       </c>
     </row>
@@ -3237,12 +3328,12 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Off (구 Disabled)</t>
+          <t>Off (이전: Disabled)</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>비활성/꺼짐</t>
+          <t>꺼짐 / 비활성 상태</t>
         </is>
       </c>
     </row>
@@ -3259,28 +3350,28 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>선택됨</t>
+          <t>선택된 상태</t>
         </is>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>v6 변경: _Hover / _Focused / _Highlight 제거 (VR/터치 환경 부재). _Active/_Disabled → _On/_Off 통합. 의미 분기는 VNT 컴포넌트 필드에서 처리.</t>
+          <t>v6 에서 바뀐 점: _Hover / _Focused / _Highlight 제거 (VR·터치 환경에서는 마우스 호버·포커스가 없음). _Active 와 _Disabled 는 _On / _Off 로 통합. "왜 꺼졌나" 같은 세부 구분은 이름 대신 VNT 설정 항목에서 처리.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>[ Direction Vocab (단문자) ]</t>
+          <t>[ 방향 약자 (한 글자) ]</t>
         </is>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Suffix</t>
+          <t>약자</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -3290,7 +3381,7 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>적용 Act</t>
+          <t>쓰는 곳</t>
         </is>
       </c>
     </row>
@@ -3302,12 +3393,12 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Left</t>
+          <t>Left (왼쪽)</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Rot, Mov</t>
+          <t>회전 · 이동</t>
         </is>
       </c>
     </row>
@@ -3319,12 +3410,12 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>Right (오른쪽)</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Rot, Mov</t>
+          <t>회전 · 이동</t>
         </is>
       </c>
     </row>
@@ -3336,12 +3427,12 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Up</t>
+          <t>Up (위)</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Rot, Mov</t>
+          <t>회전 · 이동</t>
         </is>
       </c>
     </row>
@@ -3353,12 +3444,12 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Down</t>
+          <t>Down (아래)</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Rot, Mov</t>
+          <t>회전 · 이동</t>
         </is>
       </c>
     </row>
@@ -3370,12 +3461,12 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Clockwise</t>
+          <t>Clockwise (시계 방향)</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Rot</t>
+          <t>회전</t>
         </is>
       </c>
     </row>
@@ -3387,26 +3478,26 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Counter-clockwise</t>
+          <t>Counter-clockwise (반시계 방향)</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Rot</t>
+          <t>회전</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>[ Audio Category ]</t>
+          <t>[ 오디오 카테고리 ]</t>
         </is>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>카테고리</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -3450,7 +3541,7 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>효과음 (UI 클릭·완료음·경고 등)</t>
+          <t>효과음 (UI 클릭·완료음·경고음 등)</t>
         </is>
       </c>
     </row>
@@ -3467,21 +3558,21 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>내레이션·더빙 (구 VO)</t>
+          <t>내레이션·더빙 (이전 이름: VO)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>[ Video Category ]</t>
+          <t>[ 비디오 카테고리 ]</t>
         </is>
       </c>
     </row>
     <row r="42" ht="22" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>카테고리</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -3508,7 +3599,7 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>시네마틱·서사 영상 클립</t>
+          <t>서사·시네마틱 영상 클립</t>
         </is>
       </c>
     </row>
@@ -3559,7 +3650,7 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>콘텐츠 진입 인트로</t>
+          <t>콘텐츠 시작 인트로</t>
         </is>
       </c>
     </row>
@@ -3576,21 +3667,21 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>콘텐츠 종료 아웃트로</t>
+          <t>콘텐츠 끝 아웃트로</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>[ PNG Role Token (T1 한정) ]</t>
+          <t>[ PNG 용도 약자 (T1 — 원본 파일에서만 사용) ]</t>
         </is>
       </c>
     </row>
     <row r="50" ht="22" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>Token</t>
+          <t>약자</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -3600,7 +3691,7 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>용도</t>
+          <t>어디 쓰이는지</t>
         </is>
       </c>
     </row>
@@ -3612,7 +3703,7 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>UI 스프라이트</t>
+          <t>UI 스프라이트 (버튼·아이콘 등)</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
@@ -3629,12 +3720,12 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Albedo / Base Color</t>
+          <t>Albedo / 기본 색상</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>3D Texture</t>
+          <t>3D 텍스처</t>
         </is>
       </c>
     </row>
@@ -3646,12 +3737,12 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Normal Map</t>
+          <t>Normal Map (표면 굴곡)</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>3D Texture</t>
+          <t>3D 텍스처</t>
         </is>
       </c>
     </row>
@@ -3663,12 +3754,12 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>Roughness Map</t>
+          <t>Roughness (거칠기)</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>3D Texture</t>
+          <t>3D 텍스처</t>
         </is>
       </c>
     </row>
@@ -3680,12 +3771,12 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>Metallic Map</t>
+          <t>Metallic (금속성)</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>3D Texture</t>
+          <t>3D 텍스처</t>
         </is>
       </c>
     </row>
@@ -3697,12 +3788,12 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>Emission Map</t>
+          <t>Emission (자체 발광)</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>3D Texture</t>
+          <t>3D 텍스처</t>
         </is>
       </c>
     </row>
@@ -3714,12 +3805,12 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>Mask Map</t>
+          <t>Mask (마스킹)</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>3D Texture</t>
+          <t>3D 텍스처</t>
         </is>
       </c>
     </row>
@@ -3731,12 +3822,12 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>Ambient Occlusion</t>
+          <t>Ambient Occlusion (음영)</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>3D Texture</t>
+          <t>3D 텍스처</t>
         </is>
       </c>
     </row>
@@ -3766,43 +3857,43 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>변환 예시 가이드 — 실측 파일 기준</t>
+          <t>실제 파일을 v6 규칙으로 바꾼 비교표</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Make Templete_20260512.make (513 노드) 의 실제 명명을 v6 로 변환. 각 행은 안티패턴 → 개선안 매핑.</t>
+          <t>실제 파일(Make Templete_20260512.make, 노드 513개)의 이름을 v6 규칙으로 바꾼 예시입니다. 각 행은 "현재 이름 → v6 이름 + 왜 바꾸는지" 입니다.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>[ Scene Container &amp; 위계 ]</t>
+          <t>[ 씬·페이지·계층 ]</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>현재</t>
+          <t>현재 이름</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>v6</t>
+          <t>v6 이름</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Tier</t>
+          <t>단계</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>변환 사유</t>
+          <t>왜 바꾸나</t>
         </is>
       </c>
     </row>
@@ -3824,7 +3915,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>예약어 유지</t>
+          <t>시스템 예약 이름 — 그대로 유지</t>
         </is>
       </c>
     </row>
@@ -3846,7 +3937,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>변경 없음 (간결·의미 명확)</t>
+          <t>이미 짧고 의미가 명확함 — 그대로 유지</t>
         </is>
       </c>
     </row>
@@ -3868,7 +3959,7 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>공백 → _, 하이픈 → _</t>
+          <t>공백·하이픈 → 언더바로 통일</t>
         </is>
       </c>
     </row>
@@ -3890,7 +3981,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>4단계 위계 평탄화</t>
+          <t>4단계 위계도 언더바로 평탄화</t>
         </is>
       </c>
     </row>
@@ -3912,7 +4003,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>공백 제거 + 의미 부여</t>
+          <t>공백 제거 + 의미 있는 이름 부여</t>
         </is>
       </c>
     </row>
@@ -3929,12 +4020,12 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>T2 인스턴스 (GLOSSARY)</t>
+          <t>T2 인스턴스 (용어집 등록)</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>숫자 시작 식별자 → 의미 슬러그</t>
+          <t>숫자로 시작하는 이름 → 의미 있는 이름으로</t>
         </is>
       </c>
     </row>
@@ -3948,22 +4039,22 @@
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>현재</t>
+          <t>현재 이름</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>v6</t>
+          <t>v6 이름</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Tier</t>
+          <t>단계</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>변환 사유</t>
+          <t>왜 바꾸나</t>
         </is>
       </c>
     </row>
@@ -4007,7 +4098,7 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>PascalCase + 축약</t>
+          <t>PascalCase + 축약형으로</t>
         </is>
       </c>
     </row>
@@ -4051,7 +4142,7 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>축약</t>
+          <t>축약형으로</t>
         </is>
       </c>
     </row>
@@ -4091,7 +4182,7 @@
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Family vocab Btn 적용</t>
+          <t>Family 약자 Btn 사용</t>
         </is>
       </c>
     </row>
@@ -4149,7 +4240,7 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Family vocab Pnl 적용</t>
+          <t>Family 약자 Pnl(패널) 사용</t>
         </is>
       </c>
     </row>
@@ -4171,7 +4262,7 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Navi → Nav 표기 일관성</t>
+          <t>Navi → Nav 로 표기 통일</t>
         </is>
       </c>
     </row>
@@ -4193,7 +4284,7 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Family vocab Logo, 변형 표시 _x4</t>
+          <t>Family 약자 Logo, 변형 표시는 _x4</t>
         </is>
       </c>
     </row>
@@ -4215,7 +4306,7 @@
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Family vocab Tip 단독</t>
+          <t>Family 약자 Tip 단독 사용</t>
         </is>
       </c>
     </row>
@@ -4237,36 +4328,36 @@
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Unity 자동 시퀀스 정규화</t>
+          <t>Unity 가 자동으로 붙인 번호를 정리</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>[ 방향 컨트롤 (sibling 단문자 vocab) ]</t>
+          <t>[ 방향이 있는 컨트롤 (형제 노드 한 글자 사용) ]</t>
         </is>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>현재</t>
+          <t>현재 이름</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>v6</t>
+          <t>v6 이름</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Tier</t>
+          <t>단계</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>변환 사유</t>
+          <t>왜 바꾸나</t>
         </is>
       </c>
     </row>
@@ -4288,7 +4379,7 @@
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>방향 prefix → suffix 단문자</t>
+          <t>방향을 앞이 아닌 뒤에 한 글자로</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4419,7 @@
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>방향 + State 결합</t>
+          <t>방향 + 상태 결합</t>
         </is>
       </c>
     </row>
@@ -4372,7 +4463,7 @@
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Highlight 제거 → Prs 대체</t>
+          <t>Highlight 약자 제거 → Prs 로 대체</t>
         </is>
       </c>
     </row>
@@ -4389,12 +4480,12 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>T2 (sibling)</t>
+          <t>T2 (형제 노드)</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>부모 RotationPanel 컨텍스트, 단문자 OK</t>
+          <t>부모(RotationPanel) 컨텍스트가 있어 한 글자만으로 OK</t>
         </is>
       </c>
     </row>
@@ -4411,7 +4502,7 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>T2 (sibling)</t>
+          <t>T2 (형제 노드)</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr"/>
@@ -4429,7 +4520,7 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>T2 (sibling)</t>
+          <t>T2 (형제 노드)</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr"/>
@@ -4447,7 +4538,7 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>T2 (sibling)</t>
+          <t>T2 (형제 노드)</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr"/>
@@ -4465,41 +4556,41 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>T2 (sibling)</t>
+          <t>T2 (형제 노드)</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>방향 단문자 + State</t>
+          <t>방향 + 상태</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>[ Text / Tooltip 인스턴스 ]</t>
+          <t>[ 텍스트·말풍선 인스턴스 ]</t>
         </is>
       </c>
     </row>
     <row r="44" ht="22" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>현재</t>
+          <t>현재 이름</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>v6</t>
+          <t>v6 이름</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Tier</t>
+          <t>단계</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>변환 사유</t>
+          <t>왜 바꾸나</t>
         </is>
       </c>
     </row>
@@ -4521,7 +4612,7 @@
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>의미 부여 (txt_ prefix 미사용, Family Txt 만)</t>
+          <t>의미 있는 이름 부여 (T2 에선 txt_ 같은 종류 약자 안 씀)</t>
         </is>
       </c>
     </row>
@@ -4543,7 +4634,7 @@
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>T2 인스턴스 prefix 폐지</t>
+          <t>T2 에서는 txt_ 같은 종류 약자 생략</t>
         </is>
       </c>
     </row>
@@ -4568,29 +4659,29 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>[ 머티리얼 (T3 시스템 파생) ]</t>
+          <t>[ 머티리얼 (T3 — 자동 생성) ]</t>
         </is>
       </c>
     </row>
     <row r="50" ht="22" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>현재</t>
+          <t>현재 이름</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>v6</t>
+          <t>v6 이름</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Tier</t>
+          <t>단계</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>변환 사유</t>
+          <t>왜 바꾸나</t>
         </is>
       </c>
     </row>
@@ -4607,7 +4698,7 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>T3 자동 파생</t>
+          <t>T3 자동 생성</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
@@ -4619,58 +4710,58 @@
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>(없음 — 263 머티리얼 distinct 19)</t>
+          <t>(현재 263개 중 의미 중복 19개)</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>mat_&lt;primary_node_slug&gt;</t>
+          <t>mat_&lt;쓰이는 노드 이름&gt;</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>T3 자동 파생</t>
+          <t>T3 자동 생성</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>사용 노드 분석</t>
+          <t>어떤 노드에 쓰이는지 분석해서 이름 부여</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>[ 애니메이션 (배열 위치가 타입 선언, prefix 없음) ]</t>
+          <t>[ 애니메이션 (애니메이션 목록에 들어가므로 종류 약자 없음) ]</t>
         </is>
       </c>
     </row>
     <row r="55" ht="22" customHeight="1">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>현재</t>
+          <t>현재 이름</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>v6</t>
+          <t>v6 이름</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Tier</t>
+          <t>단계</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>변환 사유</t>
+          <t>왜 바꾸나</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>new Clip (btn_start, scale)</t>
+          <t>new Clip (btn_start, 크기)</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
@@ -4680,19 +4771,19 @@
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>(animations)</t>
+          <t>(애니메이션)</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Target + Act</t>
+          <t>대상 + 동작</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>new Clip (3D Model, rotation)</t>
+          <t>new Clip (3D Model, 회전)</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
@@ -4702,19 +4793,19 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>(animations)</t>
+          <t>(애니메이션)</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>Target + Act + Dir</t>
+          <t>대상 + 동작 + 방향</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>new Clip1 (3D Model, rotation)</t>
+          <t>new Clip1 (3D Model, 회전)</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
@@ -4724,7 +4815,7 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>(animations)</t>
+          <t>(애니메이션)</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr"/>
@@ -4732,7 +4823,7 @@
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>new Clip2 (3D Model, rotation)</t>
+          <t>new Clip2 (3D Model, 회전)</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
@@ -4742,7 +4833,7 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>(animations)</t>
+          <t>(애니메이션)</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr"/>
@@ -4750,7 +4841,7 @@
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>new Clip3 (3D Model, rotation)</t>
+          <t>new Clip3 (3D Model, 회전)</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr">
@@ -4760,7 +4851,7 @@
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>(animations)</t>
+          <t>(애니메이션)</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr"/>
@@ -4768,7 +4859,7 @@
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>new Clip4 (3D Model, scl+mov)</t>
+          <t>new Clip4 (3D Model, 크기+이동)</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
@@ -4778,19 +4869,19 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>(animations)</t>
+          <t>(애니메이션)</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Compound Zoom In</t>
+          <t>Zoom In 합친 형태</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>new Clip5 (3D Model, scale)</t>
+          <t>new Clip5 (3D Model, 크기)</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
@@ -4800,12 +4891,12 @@
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>(animations)</t>
+          <t>(애니메이션)</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>Compound Zoom Out</t>
+          <t>Zoom Out 합친 형태</t>
         </is>
       </c>
     </row>
@@ -4823,59 +4914,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B48"/>
+  <dimension ref="A1:B50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="64" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Validation Checklist (.make 익스포트 전, v6)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>[ T1 — Source Asset Filesystem ]</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>검증 항목</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
+          <t>내보내기 전에 확인할 항목 (v6 체크리스트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>.make 파일을 만들기 전에 한 번씩 확인하세요. 모든 항목에 ✓ 가 들어가면 v6 규칙을 잘 따른 파일입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>[ T1 — 원본 파일 ]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>확인 항목</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>체크 [✓]</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>파일명에 공백 없음</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>구분자는 _ 만 (하이픈 0건)</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>토큰별 PascalCase</t>
+          <t>파일 이름에 공백이 없는가</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr"/>
@@ -4883,7 +4965,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Variant _NN 2자리 고정</t>
+          <t>구분자가 언더바 _ 만 쓰이는가 (하이픈 - 없음)</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr"/>
@@ -4891,7 +4973,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Version marker _v&lt;NN&gt; 는 옵션·소스 파일에만</t>
+          <t>단어마다 첫 글자가 대문자인가 (PascalCase)</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr"/>
@@ -4899,7 +4981,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>확장자가 타입 선언 시 이름에 타입 토큰 중복 없음</t>
+          <t>변형 번호가 두 자리인가 (_01, _02)</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr"/>
@@ -4907,7 +4989,7 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>PNG Role 토큰 (Sprite/ALB/NRM/...) 필수</t>
+          <t>버전 표시 _v01 은 원본 파일에만 쓰이는가</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr"/>
@@ -4915,7 +4997,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Audio 카테고리 (BGM/SFX/NAR) 첫 토큰, _ 로 desc 구분</t>
+          <t>확장자가 알려주는 종류를 이름에 또 적지 않았는가</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr"/>
@@ -4923,7 +5005,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Video 카테고리 (CUT/TUT/LOOP/INTRO/OUTRO) 첫 토큰, _ 로 desc 구분</t>
+          <t>PNG 에 용도 약자 (Sprite/ALB/NRM/...) 가 있는가</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr"/>
@@ -4931,7 +5013,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>자식 부위 FBX 는 부모 이름 포함</t>
+          <t>오디오 카테고리 (BGM/SFX/NAR) 가 맨 앞에 _ 와 함께 있는가</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr"/>
@@ -4939,50 +5021,50 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>영문 전용 (한글 파일명 0건)</t>
+          <t>비디오 카테고리 (CUT/TUT/LOOP/INTRO/OUTRO) 가 맨 앞에 _ 와 함께 있는가</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr"/>
     </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>자식 부품 FBX 에 부모 이름이 포함되어 있는가</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr"/>
+    </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>[ T2 — Instance ]</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>검증 항목</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>한글 파일명이 없는가 (영문만)</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>[ T2 — Make Editor 인스턴스 ]</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>확인 항목</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>체크 [✓]</t>
         </is>
       </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>T2 인스턴스에 kind prefix (mdl_/img_/txt_/aud_ 등) 0건</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>모든 인스턴스명 PascalCase</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>확장자 박제 0건 (*.png/*.fbx 노드명 없음)</t>
+          <t>종류 약자 (mdl_/img_/txt_/aud_ 등) 가 없는가</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr"/>
@@ -4990,7 +5072,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>구분자 단일 _ 만 (이중 __ 0건, 하이픈 0건)</t>
+          <t>모든 인스턴스명이 PascalCase 로 적혀 있는가</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr"/>
@@ -4998,7 +5080,7 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>State suffix 는 v6 vocab (_Def/_Prs/_On/_Off/_Sel) 내</t>
+          <t>이름 끝에 확장자 (.png/.fbx 등) 가 안 붙어 있는가</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr"/>
@@ -5006,7 +5088,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Direction suffix 는 v6 vocab (_L/_R/_U/_D/_CW/_CCW) 내</t>
+          <t>구분자가 언더바 _ 하나만 쓰이는가 (이중 __ 없음, 하이픈 없음)</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr"/>
@@ -5014,7 +5096,7 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>단문자 sibling 은 닫힌 vocab 부모 컨텍스트에서만 사용</t>
+          <t>상태 약자가 정해진 5개 (_Def/_Prs/_On/_Off/_Sel) 안에 있는가</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr"/>
@@ -5022,7 +5104,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>UI Family vocab (GNB/LNB/Btn/Nav/Pnl/...) 적용 권장</t>
+          <t>방향 약자가 정해진 6개 (_L/_R/_U/_D/_CW/_CCW) 안에 있는가</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr"/>
@@ -5030,50 +5112,50 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>4단계 위계는 _ 로 평탄화 (Contents_3_1_1_2)</t>
+          <t>한 글자 형제 노드는 정해진 4방향 같은 묶음에서만 쓰이는가</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr"/>
     </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>UI 종류 약자 (GNB/LNB/Btn/Nav/Pnl/...) 를 사용했는가 (권장)</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr"/>
+    </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>[ Animation ]</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>검증 항목</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>4단계 위계가 하이픈 대신 언더바로 적혀 있는가 (Contents_3_1_1_2)</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>[ 애니메이션 ]</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>확인 항목</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>체크 [✓]</t>
         </is>
       </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>애니메이션명에 prefix 없음 (&lt;Target&gt;_&lt;Act&gt;[_&lt;Dir&gt;] 패턴)</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>Action 토큰이 v6 vocab (Rot/Scl/Mov/Clr/Op 또는 ZI/ZO/FI/FO/Tx/Pop) 내</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>다중 속성 클립 토큰 순서 결정론적 (Rot → Scl → Mov → Clr → Op)</t>
+          <t>애니메이션 이름이 &lt;대상&gt;_&lt;동작&gt;[_&lt;방향&gt;] 형태인가</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr"/>
@@ -5081,50 +5163,50 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>'new Clip' 패턴 (Unity 기본값) 0건</t>
+          <t>동작 약자가 정해진 단어 (Rot/Scl/Mov/Clr/Op 또는 ZI/ZO/FI/FO/Tx/Pop) 안에 있는가</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr"/>
     </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>여러 속성이 섞일 때 순서가 회전→크기→이동→색상→투명도 인가</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr"/>
+    </row>
     <row r="36">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t>[ T3 — System-Derived ]</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="22" customHeight="1">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>검증 항목</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>'new Clip' 같은 Unity 기본값 이름이 남아 있지 않은가</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>[ T3 — 자동 생성 객체 ]</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>확인 항목</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>체크 [✓]</t>
         </is>
       </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
-        <is>
-          <t>머티리얼명에 (Instance) 사슬 0건</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
-        <is>
-          <t>머티리얼 definition 만 의미 있는 이름</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>Texture 채널 suffix (_albedo/_normal/...) 명시</t>
+          <t>머티리얼 이름에 (Instance) 가 반복되어 있지 않은가</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr"/>
@@ -5132,50 +5214,50 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Mesh·텍스처 객체 prefix (mesh_/tex_) 유지</t>
+          <t>머티리얼은 원본 정의만 의미 있는 이름인가</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr"/>
     </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>텍스처 끝 약자 (_albedo/_normal 등) 가 명시되어 있는가</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr"/>
+    </row>
     <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>[ ID·Path·Privacy ]</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="22" customHeight="1">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>검증 항목</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="inlineStr">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Mesh·텍스처 객체에 종류 약자 (mesh_/tex_) 가 유지되는가</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>[ ID·경로·개인정보 ]</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>확인 항목</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>체크 [✓]</t>
         </is>
       </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t>모든 ResourceID 가 UUID v4 포맷</t>
-        </is>
-      </c>
-      <c r="B45" s="5" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
-        <is>
-          <t>ResourceID 글로벌 유일 (중복 0건)</t>
-        </is>
-      </c>
-      <c r="B46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>공유본 OriginPath 에 사용자 홈 경로 없음 (C:\Users\, /home/)</t>
+          <t>모든 ResourceID 가 UUID v4 형식인가</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr"/>
@@ -5183,12 +5265,31 @@
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>작성자 식별 정보 누설 없음</t>
+          <t>ResourceID 가 파일 전체에서 중복되지 않는가</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr"/>
     </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>외부 공유본의 OriginPath 에 사용자 홈 경로 (C:\Users\, /home/) 가 없는가</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>작성자 식별 정보 (이메일·계정명 등) 가 누설되지 않는가</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:B3"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5202,23 +5303,23 @@
   <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>안티패턴 일람 — 실측 파일 기준</t>
+          <t>이렇게 쓰면 안 되는 예시</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Make Templete_20260512.make 분석에서 발견된 안티패턴. 모두 v6 검증에서 차단.</t>
+          <t>실제 파일(Make Templete_20260512.make) 분석에서 찾은 잘못된 이름들입니다. v6 규칙에서는 모두 막거나 자동으로 고쳐집니다.</t>
         </is>
       </c>
     </row>
@@ -5235,7 +5336,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>v6 정정</t>
+          <t>v6 에서는</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -5247,7 +5348,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>노드명에 .png/.fbx 확장자 박제</t>
+          <t>노드 이름에 .png/.fbx 같은 확장자가 붙어 있음</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -5262,14 +5363,14 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Make Editor 아이콘이 타입 표현</t>
+          <t>Make Editor 아이콘이 종류를 알려주므로 확장자 불필요</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>공백 포함 노드명</t>
+          <t>공백이 들어간 노드 이름</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -5284,14 +5385,14 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>공백 → _ 또는 의미 부여</t>
+          <t>공백을 언더바 _ 로 바꾸거나 의미 있는 이름으로</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>(Instance) 사슬 머티리얼</t>
+          <t>(Instance) 가 계속 반복된 머티리얼 이름</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -5301,19 +5402,19 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>mat_unlit_opaque (T3 정규화)</t>
+          <t>mat_unlit_opaque (T3 자동 정리)</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>임포트 시 instance chain 제거</t>
+          <t>내보낼 때 자동으로 instance 사슬 제거</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>이미지 이름이 UUID 문자열</t>
+          <t>이미지 이름이 알 수 없는 UUID 문자열</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -5323,19 +5424,19 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>img_logox4 (Tier C 파생)</t>
+          <t>img_logox4 (자동 생성)</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>ResourceID 별도, 이름은 의미</t>
+          <t>UUID 는 ID 로만 쓰고, 이름은 의미 있게</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>'new Clip*' 기본 애니메이션</t>
+          <t>'new Clip' 같은 Unity 기본값 애니메이션 이름</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -5350,14 +5451,14 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Unity 기본값 차단</t>
+          <t>Unity 기본값 그대로 두지 말 것</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>숫자 시작 노드명</t>
+          <t>숫자로 시작하는 노드 이름</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -5367,12 +5468,12 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Cupcake (GLOSSARY)</t>
+          <t>Cupcake (용어집에 등록)</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>식별자 정규식 위반</t>
+          <t>이름은 영문 글자로 시작</t>
         </is>
       </c>
     </row>
@@ -5394,14 +5495,14 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>정규화·축약</t>
+          <t>정정 + 축약형으로</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>하이픈 식별자</t>
+          <t>하이픈 - 이 들어간 이름</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -5416,14 +5517,14 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>하이픈 명시 금지</t>
+          <t>하이픈은 사용 금지</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>로컬 절대경로 OriginPath</t>
+          <t>OriginPath 에 작성자 PC 경로가 그대로 남음</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -5433,19 +5534,19 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>&lt;HOME&gt;/... 또는 OriginPath 제거</t>
+          <t>&lt;HOME&gt;/... 또는 OriginPath 자체 제거</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>정보 누설 방지</t>
+          <t>개인정보·환경 정보 누설 방지</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>한글 폴더 경로</t>
+          <t>폴더 경로에 한글이 들어감</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -5460,36 +5561,36 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>ASCII + GLOSSARY</t>
+          <t>영문으로 통일, 한글 용어는 용어집에</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>동일 노드명 sibling 대량 반복</t>
+          <t>같은 이름이 형제 노드에 대량 중복</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>GNB_Active.png ×44</t>
+          <t>GNB_Active.png 가 44번 반복</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>GNB_On (parent 가 unique 화)</t>
+          <t>GNB_On (부모 이름으로 구별)</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>트리 컨텍스트 활용</t>
+          <t>부모-자식 트리 컨텍스트로 구별</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Sprite 토큰 부재 (UI vs 3D 텍스처 혼동)</t>
+          <t>PNG 용도 약자가 빠짐 (UI 인지 3D 텍스처인지 모름)</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -5504,7 +5605,7 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>PNG 용도 명시</t>
+          <t>PNG 는 어디 쓰이는지 약자로 명시</t>
         </is>
       </c>
     </row>

</xml_diff>